<commit_message>
latest Code for Hungary
</commit_message>
<xml_diff>
--- a/Data/testDataHungry.xlsx
+++ b/Data/testDataHungry.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1145" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1149" uniqueCount="231">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -301,7 +301,7 @@
     <t>Test_1</t>
   </si>
   <si>
-    <t>Test failed for 'Zemlak Dangelo' Employee: Errors and AlertsErrorsAlertsNational IDs (Row 1)This national identifier you entered is already in use. Verify that the information is accurate.National IDs (Row 2)This national identifier you entered is already in use. Verify that the information is accurate. &amp; find failed Screenshot Path:-&gt;H:\WorkdaySuite_Playwright_MK/WorkdayFailedScreenshot/2025-03-25T07-32-16-202Z.png</t>
+    <t>Test failed for 'Brock Kulas' Employee:{undefined}TypeError: Cannot read properties of undefined (reading 'toLowerCase')</t>
   </si>
   <si>
     <t>Failed</t>
@@ -313,10 +313,10 @@
     <t>Hungary</t>
   </si>
   <si>
-    <t>Dangelo</t>
-  </si>
-  <si>
-    <t>Zemlak</t>
+    <t>Brock</t>
+  </si>
+  <si>
+    <t>Kulas</t>
   </si>
   <si>
     <t>(061)2123123</t>
@@ -404,7 +404,7 @@
     <t>Social Security</t>
   </si>
   <si>
-    <t>666666120</t>
+    <t>666666150</t>
   </si>
   <si>
     <t>01/01/2000</t>
@@ -473,6 +473,18 @@
     <t>Test_2</t>
   </si>
   <si>
+    <t xml:space="preserve">Test failed for 'Ottilie Kuphal' Employee:{10698281}TimeoutError: locator.click: Timeout 30000ms exceeded.
+Call log:
+  [2m- waiting for getByRole('button', { name: 'Approve' })[22m
+</t>
+  </si>
+  <si>
+    <t>Miguel</t>
+  </si>
+  <si>
+    <t>Prohaska</t>
+  </si>
+  <si>
     <t>I</t>
   </si>
   <si>
@@ -497,7 +509,7 @@
     <t>Social Security (TAJ) Number</t>
   </si>
   <si>
-    <t>666666121</t>
+    <t>666966123</t>
   </si>
   <si>
     <t>Female</t>
@@ -1645,7 +1657,7 @@
       </c>
       <c r="K2" s="19">
         <f t="shared" ref="K2:K15" si="0">TODAY()-31</f>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L2" s="20" t="s">
         <v>98</v>
@@ -1688,7 +1700,7 @@
       </c>
       <c r="Y2" s="19">
         <f t="shared" ref="Y2:Y15" si="1">K2</f>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z2" s="18" t="s">
         <v>113</v>
@@ -1722,11 +1734,11 @@
       </c>
       <c r="AJ2" s="31">
         <f>TODAY()+365</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AK2" s="31">
         <f t="shared" ref="AK2:AK15" si="2">Y2+90</f>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL2" s="18" t="s">
         <v>120</v>
@@ -1764,15 +1776,15 @@
       </c>
       <c r="AW2" s="33">
         <f t="shared" ref="AW2:AW15" si="4">Y2-1</f>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX2" s="33">
         <f t="shared" ref="AX2:AX15" si="5">Y2-1</f>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY2" s="34">
         <f t="shared" ref="AY2:AY7" si="6">AJ2</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AZ2" s="24" t="s">
         <v>98</v>
@@ -1796,7 +1808,7 @@
         <v>132</v>
       </c>
       <c r="BG2" s="36">
-        <v>5555000018</v>
+        <v>5555000040</v>
       </c>
       <c r="BH2" s="25">
         <v>36526</v>
@@ -1923,14 +1935,24 @@
       <c r="A3" t="s">
         <v>151</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="13"/>
+      <c r="B3" s="12" t="s">
+        <v>152</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>96</v>
+      </c>
       <c r="D3" s="14" t="s">
         <v>97</v>
       </c>
       <c r="E3" s="15" t="s">
         <v>98</v>
       </c>
+      <c r="F3" t="s">
+        <v>153</v>
+      </c>
+      <c r="G3" t="s">
+        <v>154</v>
+      </c>
       <c r="H3" s="17" t="s">
         <v>101</v>
       </c>
@@ -1942,7 +1964,7 @@
       </c>
       <c r="K3" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L3" s="20" t="s">
         <v>98</v>
@@ -1951,13 +1973,13 @@
         <v>104</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O3" s="22" t="s">
         <v>106</v>
       </c>
       <c r="P3" s="43" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="Q3" s="18">
         <v>123</v>
@@ -1985,7 +2007,7 @@
       </c>
       <c r="Y3" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z3" s="18" t="s">
         <v>113</v>
@@ -1994,13 +2016,13 @@
         <v>114</v>
       </c>
       <c r="AB3" s="44" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="AC3" s="39" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="AD3" s="45" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="AE3" s="20">
         <v>846</v>
@@ -2012,7 +2034,7 @@
         <v>10</v>
       </c>
       <c r="AH3" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="AI3" s="20" t="s">
         <v>119</v>
@@ -2022,7 +2044,7 @@
       </c>
       <c r="AK3" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL3" s="18" t="s">
         <v>120</v>
@@ -2031,7 +2053,7 @@
         <v>121</v>
       </c>
       <c r="AN3" s="39" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="AO3" s="18" t="s">
         <v>123</v>
@@ -2043,7 +2065,7 @@
         <v>124</v>
       </c>
       <c r="AR3" s="29" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AS3" s="25" t="s">
         <v>114</v>
@@ -2060,11 +2082,11 @@
       </c>
       <c r="AW3" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX3" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY3" s="34">
         <f t="shared" si="6"/>
@@ -2074,10 +2096,10 @@
         <v>98</v>
       </c>
       <c r="BA3" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB3" s="35" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="BC3" s="25">
         <v>36526</v>
@@ -2092,7 +2114,7 @@
         <v>132</v>
       </c>
       <c r="BG3" s="36">
-        <v>5555000019</v>
+        <v>5554000021</v>
       </c>
       <c r="BH3" s="25">
         <v>36526</v>
@@ -2104,7 +2126,7 @@
         <v>133</v>
       </c>
       <c r="BK3" s="29" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="BL3" s="37">
         <v>32875</v>
@@ -2143,7 +2165,7 @@
         <v>139</v>
       </c>
       <c r="BX3" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY3" s="24" t="s">
         <v>141</v>
@@ -2188,26 +2210,26 @@
         <v>98</v>
       </c>
       <c r="CM3" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN3" s="24" t="s">
         <v>150</v>
       </c>
       <c r="CO3" s="30" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="CP3" s="30" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="CQ3" s="42" t="s">
         <v>110</v>
       </c>
       <c r="CR3" s="48">
         <f>TODAY()-1500</f>
-        <v>44240</v>
+        <v>44250</v>
       </c>
       <c r="CS3" s="30" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="CT3" s="41">
         <v>1234022</v>
@@ -2219,10 +2241,10 @@
     </row>
     <row r="4" ht="14.5" customHeight="1" spans="1:100" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>98</v>
@@ -2240,7 +2262,7 @@
       </c>
       <c r="K4" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L4" s="20" t="s">
         <v>98</v>
@@ -2283,22 +2305,22 @@
       </c>
       <c r="Y4" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z4" s="18" t="s">
         <v>113</v>
       </c>
       <c r="AA4" s="27" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="AB4" s="32" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="AC4" s="29" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="AD4" s="30" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="AE4" s="20">
         <v>846</v>
@@ -2310,7 +2332,7 @@
         <v>10</v>
       </c>
       <c r="AH4" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="AI4" s="20" t="s">
         <v>119</v>
@@ -2320,16 +2342,16 @@
       </c>
       <c r="AK4" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL4" s="18" t="s">
         <v>120</v>
       </c>
       <c r="AM4" s="29" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AN4" s="39" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AO4" s="18" t="s">
         <v>123</v>
@@ -2358,11 +2380,11 @@
       </c>
       <c r="AW4" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX4" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY4" s="50" t="str">
         <f t="shared" si="6"/>
@@ -2372,10 +2394,10 @@
         <v>98</v>
       </c>
       <c r="BA4" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB4" s="35" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="BC4" s="25">
         <v>36526</v>
@@ -2402,7 +2424,7 @@
         <v>133</v>
       </c>
       <c r="BK4" s="29" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="BL4" s="37">
         <v>32875</v>
@@ -2441,7 +2463,7 @@
         <v>139</v>
       </c>
       <c r="BX4" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY4" s="24" t="s">
         <v>141</v>
@@ -2486,16 +2508,16 @@
         <v>98</v>
       </c>
       <c r="CM4" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN4" s="24" t="s">
         <v>150</v>
       </c>
       <c r="CO4" s="32" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="CP4" s="30" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="CQ4" s="42" t="s">
         <v>110</v>
@@ -2504,7 +2526,7 @@
         <v>31048</v>
       </c>
       <c r="CS4" s="30" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="CT4" s="41">
         <v>1234011</v>
@@ -2516,10 +2538,10 @@
     </row>
     <row r="5" ht="14.5" customHeight="1" spans="1:99" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E5" s="15" t="s">
         <v>98</v>
@@ -2537,7 +2559,7 @@
       </c>
       <c r="K5" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L5" s="20" t="s">
         <v>98</v>
@@ -2546,13 +2568,13 @@
         <v>104</v>
       </c>
       <c r="N5" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O5" s="22" t="s">
         <v>106</v>
       </c>
       <c r="P5" s="43" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="Q5" s="18">
         <v>123</v>
@@ -2580,19 +2602,19 @@
       </c>
       <c r="Y5" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z5" s="18" t="s">
         <v>113</v>
       </c>
       <c r="AA5" s="27" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AB5" s="44" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AC5" s="51" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="AD5" s="30" t="s">
         <v>117</v>
@@ -2607,27 +2629,27 @@
         <v>40</v>
       </c>
       <c r="AH5" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="AI5" s="20" t="s">
         <v>119</v>
       </c>
       <c r="AJ5" s="31">
         <f>TODAY()+365</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AK5" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL5" s="18" t="s">
         <v>120</v>
       </c>
       <c r="AM5" s="29" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AN5" s="51" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AO5" s="18" t="s">
         <v>123</v>
@@ -2656,24 +2678,24 @@
       </c>
       <c r="AW5" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX5" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY5" s="34">
         <f t="shared" si="6"/>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AZ5" s="24" t="s">
         <v>98</v>
       </c>
       <c r="BA5" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB5" s="35" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="BC5" s="25">
         <v>36526</v>
@@ -2739,7 +2761,7 @@
         <v>139</v>
       </c>
       <c r="BX5" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY5" s="24" t="s">
         <v>141</v>
@@ -2784,7 +2806,7 @@
         <v>98</v>
       </c>
       <c r="CM5" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN5" s="24" t="s">
         <v>150</v>
@@ -2813,10 +2835,10 @@
     </row>
     <row r="6" ht="14.5" customHeight="1" spans="1:99" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E6" s="15" t="s">
         <v>98</v>
@@ -2834,7 +2856,7 @@
       </c>
       <c r="K6" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L6" s="20" t="s">
         <v>98</v>
@@ -2843,13 +2865,13 @@
         <v>104</v>
       </c>
       <c r="N6" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O6" s="22" t="s">
         <v>106</v>
       </c>
       <c r="P6" s="23" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="Q6" s="18">
         <v>123</v>
@@ -2877,22 +2899,22 @@
       </c>
       <c r="Y6" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z6" s="18" t="s">
         <v>113</v>
       </c>
       <c r="AA6" s="27" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="AB6" s="54" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="AC6" s="51" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="AD6" s="30" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="AE6" s="20">
         <v>846</v>
@@ -2914,16 +2936,16 @@
       </c>
       <c r="AK6" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL6" s="18" t="s">
         <v>120</v>
       </c>
       <c r="AM6" s="29" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AN6" s="51" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AO6" s="18" t="s">
         <v>123</v>
@@ -2952,11 +2974,11 @@
       </c>
       <c r="AW6" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX6" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY6" s="34">
         <f t="shared" si="6"/>
@@ -2966,10 +2988,10 @@
         <v>98</v>
       </c>
       <c r="BA6" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB6" s="35" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="BC6" s="25">
         <v>36526</v>
@@ -2996,7 +3018,7 @@
         <v>133</v>
       </c>
       <c r="BK6" s="29" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="BL6" s="37">
         <v>32875</v>
@@ -3035,7 +3057,7 @@
         <v>139</v>
       </c>
       <c r="BX6" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY6" s="24" t="s">
         <v>141</v>
@@ -3080,16 +3102,16 @@
         <v>98</v>
       </c>
       <c r="CM6" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN6" s="24" t="s">
         <v>150</v>
       </c>
       <c r="CO6" s="32" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="CP6" s="30" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="CQ6" s="42" t="s">
         <v>110</v>
@@ -3098,7 +3120,7 @@
         <v>31048</v>
       </c>
       <c r="CS6" s="30" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="CT6" s="41">
         <v>1234015</v>
@@ -3109,10 +3131,10 @@
     </row>
     <row r="7" ht="14.5" customHeight="1" spans="1:99" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E7" s="15" t="s">
         <v>98</v>
@@ -3130,7 +3152,7 @@
       </c>
       <c r="K7" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L7" s="20" t="s">
         <v>98</v>
@@ -3139,13 +3161,13 @@
         <v>104</v>
       </c>
       <c r="N7" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O7" s="22" t="s">
         <v>106</v>
       </c>
       <c r="P7" s="49" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="Q7" s="18">
         <v>123</v>
@@ -3173,19 +3195,19 @@
       </c>
       <c r="Y7" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z7" s="18" t="s">
         <v>113</v>
       </c>
       <c r="AA7" s="27" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="AB7" s="44" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AC7" s="51" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="AD7" s="30" t="s">
         <v>117</v>
@@ -3200,27 +3222,27 @@
         <v>40</v>
       </c>
       <c r="AH7" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="AI7" s="20" t="s">
         <v>119</v>
       </c>
       <c r="AJ7" s="31">
         <f>TODAY()+365</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AK7" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL7" s="18" t="s">
         <v>120</v>
       </c>
       <c r="AM7" s="29" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AN7" s="51" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AO7" s="18" t="s">
         <v>123</v>
@@ -3249,24 +3271,24 @@
       </c>
       <c r="AW7" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX7" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY7" s="34">
         <f t="shared" si="6"/>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AZ7" s="24" t="s">
         <v>98</v>
       </c>
       <c r="BA7" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB7" s="35" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="BC7" s="25">
         <v>36526</v>
@@ -3332,7 +3354,7 @@
         <v>139</v>
       </c>
       <c r="BX7" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY7" s="24" t="s">
         <v>141</v>
@@ -3377,7 +3399,7 @@
         <v>98</v>
       </c>
       <c r="CM7" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN7" s="24" t="s">
         <v>150</v>
@@ -3406,10 +3428,10 @@
     </row>
     <row r="8" ht="14.5" customHeight="1" spans="1:99" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E8" s="15" t="s">
         <v>98</v>
@@ -3427,7 +3449,7 @@
       </c>
       <c r="K8" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L8" s="20" t="s">
         <v>98</v>
@@ -3436,13 +3458,13 @@
         <v>104</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O8" s="22" t="s">
         <v>106</v>
       </c>
       <c r="P8" s="49" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="Q8" s="18">
         <v>123</v>
@@ -3470,22 +3492,22 @@
       </c>
       <c r="Y8" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z8" s="18" t="s">
         <v>113</v>
       </c>
       <c r="AA8" s="27" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="AB8" s="54" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="AC8" s="51" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="AD8" s="30" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="AE8" s="20">
         <v>846</v>
@@ -3507,16 +3529,16 @@
       </c>
       <c r="AK8" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL8" s="18" t="s">
         <v>120</v>
       </c>
       <c r="AM8" s="29" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AN8" s="51" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AO8" s="18" t="s">
         <v>123</v>
@@ -3545,11 +3567,11 @@
       </c>
       <c r="AW8" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX8" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY8" s="34" t="s">
         <v>114</v>
@@ -3558,10 +3580,10 @@
         <v>98</v>
       </c>
       <c r="BA8" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB8" s="35" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="BC8" s="25">
         <v>36526</v>
@@ -3588,7 +3610,7 @@
         <v>133</v>
       </c>
       <c r="BK8" s="29" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="BL8" s="37">
         <v>32875</v>
@@ -3627,7 +3649,7 @@
         <v>139</v>
       </c>
       <c r="BX8" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY8" s="24" t="s">
         <v>141</v>
@@ -3672,26 +3694,26 @@
         <v>98</v>
       </c>
       <c r="CM8" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN8" s="24" t="s">
         <v>150</v>
       </c>
       <c r="CO8" s="30" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="CP8" s="30" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="CQ8" s="42" t="s">
         <v>110</v>
       </c>
       <c r="CR8" s="48">
         <f>TODAY()-1500</f>
-        <v>44240</v>
+        <v>44250</v>
       </c>
       <c r="CS8" s="30" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="CT8" s="41">
         <v>1234015</v>
@@ -3702,10 +3724,10 @@
     </row>
     <row r="9" ht="14.5" customHeight="1" spans="1:99" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E9" s="15" t="s">
         <v>98</v>
@@ -3723,7 +3745,7 @@
       </c>
       <c r="K9" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L9" s="20" t="s">
         <v>98</v>
@@ -3732,13 +3754,13 @@
         <v>104</v>
       </c>
       <c r="N9" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O9" s="22" t="s">
         <v>106</v>
       </c>
       <c r="P9" s="49" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="Q9" s="18">
         <v>123</v>
@@ -3766,19 +3788,19 @@
       </c>
       <c r="Y9" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z9" s="18" t="s">
         <v>113</v>
       </c>
       <c r="AA9" s="27" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="AB9" s="44" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AC9" s="51" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="AD9" s="30" t="s">
         <v>117</v>
@@ -3793,27 +3815,27 @@
         <v>40</v>
       </c>
       <c r="AH9" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="AI9" s="20" t="s">
         <v>119</v>
       </c>
       <c r="AJ9" s="31">
         <f>TODAY()+365</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AK9" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL9" s="18" t="s">
         <v>120</v>
       </c>
       <c r="AM9" s="29" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AN9" s="51" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AO9" s="18" t="s">
         <v>123</v>
@@ -3842,24 +3864,24 @@
       </c>
       <c r="AW9" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX9" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY9" s="34">
         <f>AJ9</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AZ9" s="24" t="s">
         <v>98</v>
       </c>
       <c r="BA9" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB9" s="35" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="BC9" s="25">
         <v>36526</v>
@@ -3925,7 +3947,7 @@
         <v>139</v>
       </c>
       <c r="BX9" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY9" s="24" t="s">
         <v>141</v>
@@ -3970,7 +3992,7 @@
         <v>98</v>
       </c>
       <c r="CM9" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN9" s="24" t="s">
         <v>150</v>
@@ -3999,7 +4021,7 @@
     </row>
     <row r="10" ht="14.5" customHeight="1" spans="1:99" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>97</v>
@@ -4020,7 +4042,7 @@
       </c>
       <c r="K10" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L10" s="20" t="s">
         <v>98</v>
@@ -4029,13 +4051,13 @@
         <v>104</v>
       </c>
       <c r="N10" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O10" s="22" t="s">
         <v>106</v>
       </c>
       <c r="P10" s="23" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="Q10" s="18">
         <v>123</v>
@@ -4063,7 +4085,7 @@
       </c>
       <c r="Y10" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z10" s="18" t="s">
         <v>113</v>
@@ -4072,13 +4094,13 @@
         <v>114</v>
       </c>
       <c r="AB10" s="54" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="AC10" s="51" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="AD10" s="30" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="AE10" s="20">
         <v>846</v>
@@ -4100,7 +4122,7 @@
       </c>
       <c r="AK10" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL10" s="18" t="s">
         <v>120</v>
@@ -4109,7 +4131,7 @@
         <v>121</v>
       </c>
       <c r="AN10" s="51" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="AO10" s="18" t="s">
         <v>123</v>
@@ -4138,11 +4160,11 @@
       </c>
       <c r="AW10" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX10" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY10" s="34" t="s">
         <v>114</v>
@@ -4151,10 +4173,10 @@
         <v>98</v>
       </c>
       <c r="BA10" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB10" s="35" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="BC10" s="25">
         <v>36526</v>
@@ -4181,7 +4203,7 @@
         <v>133</v>
       </c>
       <c r="BK10" s="29" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="BL10" s="37">
         <v>32875</v>
@@ -4220,7 +4242,7 @@
         <v>139</v>
       </c>
       <c r="BX10" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY10" s="24" t="s">
         <v>141</v>
@@ -4265,7 +4287,7 @@
         <v>98</v>
       </c>
       <c r="CM10" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN10" s="24" t="s">
         <v>150</v>
@@ -4294,7 +4316,7 @@
     </row>
     <row r="11" ht="14.5" customHeight="1" spans="1:99" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D11" s="14" t="s">
         <v>97</v>
@@ -4315,7 +4337,7 @@
       </c>
       <c r="K11" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L11" s="20" t="s">
         <v>98</v>
@@ -4324,13 +4346,13 @@
         <v>104</v>
       </c>
       <c r="N11" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O11" s="22" t="s">
         <v>106</v>
       </c>
       <c r="P11" s="49" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="Q11" s="18">
         <v>123</v>
@@ -4358,7 +4380,7 @@
       </c>
       <c r="Y11" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z11" s="18" t="s">
         <v>113</v>
@@ -4367,10 +4389,10 @@
         <v>114</v>
       </c>
       <c r="AB11" s="44" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AC11" s="51" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="AD11" s="30" t="s">
         <v>117</v>
@@ -4385,18 +4407,18 @@
         <v>40</v>
       </c>
       <c r="AH11" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="AI11" s="20" t="s">
         <v>119</v>
       </c>
       <c r="AJ11" s="31">
         <f>TODAY()+365</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AK11" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL11" s="18" t="s">
         <v>120</v>
@@ -4405,7 +4427,7 @@
         <v>121</v>
       </c>
       <c r="AN11" s="51" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="AO11" s="18" t="s">
         <v>123</v>
@@ -4434,24 +4456,24 @@
       </c>
       <c r="AW11" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX11" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY11" s="34">
         <f>AJ11</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AZ11" s="24" t="s">
         <v>98</v>
       </c>
       <c r="BA11" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB11" s="35" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="BC11" s="25">
         <v>36526</v>
@@ -4517,7 +4539,7 @@
         <v>139</v>
       </c>
       <c r="BX11" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY11" s="24" t="s">
         <v>141</v>
@@ -4562,26 +4584,26 @@
         <v>98</v>
       </c>
       <c r="CM11" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN11" s="24" t="s">
         <v>150</v>
       </c>
       <c r="CO11" s="30" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="CP11" s="30" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="CQ11" s="42" t="s">
         <v>110</v>
       </c>
       <c r="CR11" s="48">
         <f>TODAY()-1500</f>
-        <v>44240</v>
+        <v>44250</v>
       </c>
       <c r="CS11" s="30" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="CT11" s="41">
         <v>1234015</v>
@@ -4592,7 +4614,7 @@
     </row>
     <row r="12" ht="14.5" customHeight="1" spans="1:99" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D12" s="14" t="s">
         <v>97</v>
@@ -4613,7 +4635,7 @@
       </c>
       <c r="K12" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L12" s="20" t="s">
         <v>98</v>
@@ -4622,13 +4644,13 @@
         <v>104</v>
       </c>
       <c r="N12" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O12" s="22" t="s">
         <v>106</v>
       </c>
       <c r="P12" s="49" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="Q12" s="18">
         <v>123</v>
@@ -4656,7 +4678,7 @@
       </c>
       <c r="Y12" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z12" s="18" t="s">
         <v>113</v>
@@ -4665,13 +4687,13 @@
         <v>114</v>
       </c>
       <c r="AB12" s="54" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="AC12" s="51" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="AD12" s="30" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="AE12" s="20">
         <v>846</v>
@@ -4693,7 +4715,7 @@
       </c>
       <c r="AK12" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL12" s="18" t="s">
         <v>120</v>
@@ -4702,7 +4724,7 @@
         <v>121</v>
       </c>
       <c r="AN12" s="51" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="AO12" s="18" t="s">
         <v>123</v>
@@ -4731,11 +4753,11 @@
       </c>
       <c r="AW12" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX12" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY12" s="34">
         <f>AJ12</f>
@@ -4745,10 +4767,10 @@
         <v>98</v>
       </c>
       <c r="BA12" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB12" s="35" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="BC12" s="25">
         <v>36526</v>
@@ -4775,7 +4797,7 @@
         <v>133</v>
       </c>
       <c r="BK12" s="29" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="BL12" s="37">
         <v>32875</v>
@@ -4814,7 +4836,7 @@
         <v>139</v>
       </c>
       <c r="BX12" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY12" s="24" t="s">
         <v>141</v>
@@ -4859,7 +4881,7 @@
         <v>98</v>
       </c>
       <c r="CM12" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN12" s="24" t="s">
         <v>150</v>
@@ -4888,10 +4910,10 @@
     </row>
     <row r="13" ht="14.5" customHeight="1" spans="1:99" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E13" s="15" t="s">
         <v>98</v>
@@ -4909,7 +4931,7 @@
       </c>
       <c r="K13" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L13" s="20" t="s">
         <v>98</v>
@@ -4918,7 +4940,7 @@
         <v>104</v>
       </c>
       <c r="N13" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O13" s="22" t="s">
         <v>106</v>
@@ -4952,19 +4974,19 @@
       </c>
       <c r="Y13" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z13" s="18" t="s">
         <v>113</v>
       </c>
       <c r="AA13" s="27" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="AB13" s="44" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AC13" s="51" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="AD13" s="30" t="s">
         <v>117</v>
@@ -4979,27 +5001,27 @@
         <v>40</v>
       </c>
       <c r="AH13" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="AI13" s="20" t="s">
         <v>119</v>
       </c>
       <c r="AJ13" s="31">
         <f>TODAY()+365</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AK13" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL13" s="18" t="s">
         <v>120</v>
       </c>
       <c r="AM13" s="29" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="AN13" s="51" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AO13" s="18" t="s">
         <v>123</v>
@@ -5028,24 +5050,24 @@
       </c>
       <c r="AW13" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX13" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY13" s="34">
         <f>AJ13</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AZ13" s="24" t="s">
         <v>98</v>
       </c>
       <c r="BA13" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB13" s="35" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="BC13" s="25">
         <v>36526</v>
@@ -5111,7 +5133,7 @@
         <v>139</v>
       </c>
       <c r="BX13" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY13" s="24" t="s">
         <v>141</v>
@@ -5156,7 +5178,7 @@
         <v>98</v>
       </c>
       <c r="CM13" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN13" s="24" t="s">
         <v>150</v>
@@ -5185,7 +5207,7 @@
     </row>
     <row r="14" ht="14.5" customHeight="1" spans="1:99" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>97</v>
@@ -5206,7 +5228,7 @@
       </c>
       <c r="K14" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L14" s="20" t="s">
         <v>98</v>
@@ -5215,13 +5237,13 @@
         <v>104</v>
       </c>
       <c r="N14" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O14" s="22" t="s">
         <v>106</v>
       </c>
       <c r="P14" s="23" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="Q14" s="18">
         <v>123</v>
@@ -5249,7 +5271,7 @@
       </c>
       <c r="Y14" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z14" s="18" t="s">
         <v>113</v>
@@ -5258,13 +5280,13 @@
         <v>114</v>
       </c>
       <c r="AB14" s="54" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="AC14" s="29" t="s">
         <v>116</v>
       </c>
       <c r="AD14" s="30" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="AE14" s="20">
         <v>846</v>
@@ -5286,7 +5308,7 @@
       </c>
       <c r="AK14" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL14" s="18" t="s">
         <v>120</v>
@@ -5295,7 +5317,7 @@
         <v>121</v>
       </c>
       <c r="AN14" s="51" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="AO14" s="18" t="s">
         <v>123</v>
@@ -5324,11 +5346,11 @@
       </c>
       <c r="AW14" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX14" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY14" s="34">
         <f>AJ14</f>
@@ -5338,10 +5360,10 @@
         <v>98</v>
       </c>
       <c r="BA14" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB14" s="35" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="BC14" s="25">
         <v>36526</v>
@@ -5368,7 +5390,7 @@
         <v>133</v>
       </c>
       <c r="BK14" s="29" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="BL14" s="37">
         <v>32875</v>
@@ -5407,7 +5429,7 @@
         <v>139</v>
       </c>
       <c r="BX14" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY14" s="24" t="s">
         <v>141</v>
@@ -5452,16 +5474,16 @@
         <v>98</v>
       </c>
       <c r="CM14" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN14" s="24" t="s">
         <v>150</v>
       </c>
       <c r="CO14" s="32" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="CP14" s="30" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="CQ14" s="42" t="s">
         <v>110</v>
@@ -5470,7 +5492,7 @@
         <v>31048</v>
       </c>
       <c r="CS14" s="30" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="CT14" s="41">
         <v>1234015</v>
@@ -5481,10 +5503,10 @@
     </row>
     <row r="15" ht="14.5" customHeight="1" spans="1:99" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E15" s="15" t="s">
         <v>98</v>
@@ -5502,7 +5524,7 @@
       </c>
       <c r="K15" s="19">
         <f t="shared" si="0"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="L15" s="20" t="s">
         <v>98</v>
@@ -5511,13 +5533,13 @@
         <v>104</v>
       </c>
       <c r="N15" s="18" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="O15" s="22" t="s">
         <v>106</v>
       </c>
       <c r="P15" s="49" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="Q15" s="18">
         <v>123</v>
@@ -5545,19 +5567,19 @@
       </c>
       <c r="Y15" s="19">
         <f t="shared" si="1"/>
-        <v>45709</v>
+        <v>45719</v>
       </c>
       <c r="Z15" s="18" t="s">
         <v>113</v>
       </c>
       <c r="AA15" s="27" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="AB15" s="44" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="AC15" s="51" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="AD15" s="30" t="s">
         <v>117</v>
@@ -5572,27 +5594,27 @@
         <v>40</v>
       </c>
       <c r="AH15" s="29" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="AI15" s="20" t="s">
         <v>119</v>
       </c>
       <c r="AJ15" s="31">
         <f>TODAY()+365</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AK15" s="31">
         <f t="shared" si="2"/>
-        <v>45799</v>
+        <v>45809</v>
       </c>
       <c r="AL15" s="18" t="s">
         <v>120</v>
       </c>
       <c r="AM15" s="29" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="AN15" s="51" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="AO15" s="18" t="s">
         <v>123</v>
@@ -5621,24 +5643,24 @@
       </c>
       <c r="AW15" s="33">
         <f t="shared" si="4"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AX15" s="33">
         <f t="shared" si="5"/>
-        <v>45708</v>
+        <v>45718</v>
       </c>
       <c r="AY15" s="34">
         <f>AJ15</f>
-        <v>46105</v>
+        <v>46115</v>
       </c>
       <c r="AZ15" s="24" t="s">
         <v>98</v>
       </c>
       <c r="BA15" s="24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="BB15" s="35" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="BC15" s="25">
         <v>36526</v>
@@ -5704,7 +5726,7 @@
         <v>139</v>
       </c>
       <c r="BX15" s="47" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="BY15" s="24" t="s">
         <v>141</v>
@@ -5749,7 +5771,7 @@
         <v>98</v>
       </c>
       <c r="CM15" s="24" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="CN15" s="24" t="s">
         <v>150</v>

</xml_diff>